<commit_message>
Updated TestData.xlsx added loginTest
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
   <si>
     <t>TestName</t>
   </si>
@@ -22,16 +22,7 @@
     <t>password</t>
   </si>
   <si>
-    <t>confirmPassword</t>
-  </si>
-  <si>
-    <t>firstName</t>
-  </si>
-  <si>
-    <t>lastName</t>
-  </si>
-  <si>
-    <t>validLoginTest</t>
+    <t>LoginTest</t>
   </si>
   <si>
     <t>test@gmail.com</t>
@@ -40,25 +31,10 @@
     <t>password1</t>
   </si>
   <si>
-    <t>invalidLoginTest</t>
-  </si>
-  <si>
-    <t>wrong@mail.com</t>
-  </si>
-  <si>
-    <t>wrongpass</t>
-  </si>
-  <si>
     <t>validSignupTest</t>
   </si>
   <si>
     <t>new@mail.com</t>
-  </si>
-  <si>
-    <t>Uma</t>
-  </si>
-  <si>
-    <t>k</t>
   </si>
   <si>
     <t>invalidSignupTest</t>
@@ -327,7 +303,6 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="14.75"/>
     <col customWidth="1" min="2" max="2" width="14.38"/>
-    <col customWidth="1" min="4" max="4" width="16.5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -340,76 +315,38 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>